<commit_message>
Daily recap, matchup updates, learning and research 2026-08-15
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-15.xlsx
+++ b/data/k-props/2026-08-15.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="99">
   <si>
     <t>date</t>
   </si>
@@ -145,21 +145,30 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Troy Melton</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Troy Melton</t>
-  </si>
-  <si>
     <t>Michael McGreevy</t>
   </si>
   <si>
     <t>St. Louis Cardinals @ Chicago Cubs</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t>Matthew Boyd</t>
   </si>
   <si>
@@ -227,6 +236,9 @@
   </si>
   <si>
     <t>Joey Cantillo</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
   <si>
     <t>Emerson Hancock</t>
@@ -877,17 +889,23 @@
       <c r="Y2">
         <v>0.9736</v>
       </c>
+      <c r="Z2">
+        <v>4</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>-1.28</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>3.22</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.1825</v>
@@ -897,6 +915,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>0.78</v>
+      </c>
+      <c r="AJ2">
+        <v>0.78</v>
+      </c>
+      <c r="AK2">
+        <v>0.78</v>
+      </c>
+      <c r="AL2">
+        <v>0.78</v>
       </c>
       <c r="AM2">
         <v>3.22</v>
@@ -907,7 +937,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>5.5</v>
@@ -978,17 +1008,23 @@
       <c r="Y3">
         <v>1.0768</v>
       </c>
+      <c r="Z3">
+        <v>4</v>
+      </c>
       <c r="AA3" t="s">
         <v>44</v>
       </c>
+      <c r="AB3">
+        <v>0.25</v>
+      </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD3">
         <v>5.75</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.2125</v>
@@ -998,6 +1034,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-1.75</v>
+      </c>
+      <c r="AJ3">
+        <v>1.75</v>
+      </c>
+      <c r="AK3">
+        <v>-1.75</v>
+      </c>
+      <c r="AL3">
+        <v>1.75</v>
       </c>
       <c r="AM3">
         <v>5.75</v>
@@ -1008,7 +1056,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>3.5</v>
@@ -1020,7 +1068,7 @@
         <v>-125</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>824644</v>
@@ -1079,17 +1127,23 @@
       <c r="Y4">
         <v>0.9668</v>
       </c>
+      <c r="Z4">
+        <v>6</v>
+      </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB4">
+        <v>0.65</v>
       </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD4">
         <v>4.15</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
         <v>0.1731</v>
@@ -1099,6 +1153,18 @@
       </c>
       <c r="AH4">
         <v>0</v>
+      </c>
+      <c r="AI4">
+        <v>1.85</v>
+      </c>
+      <c r="AJ4">
+        <v>1.85</v>
+      </c>
+      <c r="AK4">
+        <v>1.85</v>
+      </c>
+      <c r="AL4">
+        <v>1.85</v>
       </c>
       <c r="AM4">
         <v>4.15</v>
@@ -1109,7 +1175,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>4.5</v>
@@ -1121,7 +1187,7 @@
         <v>-106</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <v>824644</v>
@@ -1180,17 +1246,23 @@
       <c r="Y5">
         <v>0.9265</v>
       </c>
+      <c r="Z5">
+        <v>2</v>
+      </c>
       <c r="AA5" t="s">
         <v>44</v>
       </c>
+      <c r="AB5">
+        <v>-0.43</v>
+      </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD5">
         <v>4.07</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
         <v>0.1644</v>
@@ -1200,6 +1272,18 @@
       </c>
       <c r="AH5">
         <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>-2.07</v>
+      </c>
+      <c r="AJ5">
+        <v>2.07</v>
+      </c>
+      <c r="AK5">
+        <v>-2.07</v>
+      </c>
+      <c r="AL5">
+        <v>2.07</v>
       </c>
       <c r="AM5">
         <v>4.07</v>
@@ -1210,7 +1294,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C6">
         <v>6.5</v>
@@ -1222,7 +1306,7 @@
         <v>105</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G6">
         <v>822775</v>
@@ -1281,17 +1365,23 @@
       <c r="Y6">
         <v>1.0898</v>
       </c>
+      <c r="Z6">
+        <v>7</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB6">
+        <v>2.08</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD6">
         <v>9.35</v>
       </c>
       <c r="AE6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="AF6">
         <v>0.3412</v>
@@ -1301,6 +1391,18 @@
       </c>
       <c r="AH6">
         <v>-0.77</v>
+      </c>
+      <c r="AI6">
+        <v>-2.35</v>
+      </c>
+      <c r="AJ6">
+        <v>2.35</v>
+      </c>
+      <c r="AK6">
+        <v>-1.58</v>
+      </c>
+      <c r="AL6">
+        <v>1.58</v>
       </c>
       <c r="AM6">
         <v>8.58</v>
@@ -1311,16 +1413,16 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G7">
         <v>822775</v>
       </c>
       <c r="H7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I7">
         <v>1.1</v>
@@ -1374,16 +1476,16 @@
         <v>1.0475</v>
       </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD7">
         <v>1.2</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
         <v>0.2198</v>
@@ -1403,7 +1505,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C8">
         <v>3.5</v>
@@ -1415,7 +1517,7 @@
         <v>-140</v>
       </c>
       <c r="F8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G8">
         <v>823184</v>
@@ -1474,17 +1576,23 @@
       <c r="Y8">
         <v>0.9007</v>
       </c>
+      <c r="Z8">
+        <v>1</v>
+      </c>
       <c r="AA8" t="s">
         <v>44</v>
       </c>
+      <c r="AB8">
+        <v>-0.75</v>
+      </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD8">
         <v>2.75</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.1277</v>
@@ -1494,6 +1602,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>-1.75</v>
+      </c>
+      <c r="AJ8">
+        <v>1.75</v>
+      </c>
+      <c r="AK8">
+        <v>-1.75</v>
+      </c>
+      <c r="AL8">
+        <v>1.75</v>
       </c>
       <c r="AM8">
         <v>2.75</v>
@@ -1504,7 +1624,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C9">
         <v>5.5</v>
@@ -1516,7 +1636,7 @@
         <v>100</v>
       </c>
       <c r="F9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>823184</v>
@@ -1575,17 +1695,23 @@
       <c r="Y9">
         <v>0.9947</v>
       </c>
+      <c r="Z9">
+        <v>7</v>
+      </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB9">
+        <v>-0.43</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD9">
         <v>5.07</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.1996</v>
@@ -1595,6 +1721,18 @@
       </c>
       <c r="AH9">
         <v>0</v>
+      </c>
+      <c r="AI9">
+        <v>1.93</v>
+      </c>
+      <c r="AJ9">
+        <v>1.93</v>
+      </c>
+      <c r="AK9">
+        <v>1.93</v>
+      </c>
+      <c r="AL9">
+        <v>1.93</v>
       </c>
       <c r="AM9">
         <v>5.07</v>
@@ -1605,7 +1743,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C10">
         <v>3.5</v>
@@ -1617,13 +1755,13 @@
         <v>-164</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G10">
         <v>823588</v>
       </c>
       <c r="H10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I10">
         <v>1.9</v>
@@ -1676,17 +1814,23 @@
       <c r="Y10">
         <v>0.9929</v>
       </c>
+      <c r="Z10">
+        <v>1</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>-1.53</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD10">
         <v>1.97</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.2113</v>
@@ -1696,6 +1840,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>-0.97</v>
+      </c>
+      <c r="AJ10">
+        <v>0.97</v>
+      </c>
+      <c r="AK10">
+        <v>-0.97</v>
+      </c>
+      <c r="AL10">
+        <v>0.97</v>
       </c>
       <c r="AM10">
         <v>1.97</v>
@@ -1706,7 +1862,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C11">
         <v>5.5</v>
@@ -1718,7 +1874,7 @@
         <v>122</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G11">
         <v>823588</v>
@@ -1777,17 +1933,23 @@
       <c r="Y11">
         <v>1.0233</v>
       </c>
+      <c r="Z11">
+        <v>7</v>
+      </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB11">
+        <v>0.29</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD11">
         <v>5.79</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.2408</v>
@@ -1797,6 +1959,18 @@
       </c>
       <c r="AH11">
         <v>0</v>
+      </c>
+      <c r="AI11">
+        <v>1.21</v>
+      </c>
+      <c r="AJ11">
+        <v>1.21</v>
+      </c>
+      <c r="AK11">
+        <v>1.21</v>
+      </c>
+      <c r="AL11">
+        <v>1.21</v>
       </c>
       <c r="AM11">
         <v>5.79</v>
@@ -1807,7 +1981,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C12">
         <v>4.5</v>
@@ -1819,7 +1993,7 @@
         <v>-115</v>
       </c>
       <c r="F12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G12">
         <v>822941</v>
@@ -1878,17 +2052,23 @@
       <c r="Y12">
         <v>0.88</v>
       </c>
+      <c r="Z12">
+        <v>3</v>
+      </c>
       <c r="AA12" t="s">
         <v>44</v>
       </c>
+      <c r="AB12">
+        <v>-1.13</v>
+      </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD12">
         <v>3.37</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.2017</v>
@@ -1898,6 +2078,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>-0.37</v>
+      </c>
+      <c r="AJ12">
+        <v>0.37</v>
+      </c>
+      <c r="AK12">
+        <v>-0.37</v>
+      </c>
+      <c r="AL12">
+        <v>0.37</v>
       </c>
       <c r="AM12">
         <v>3.37</v>
@@ -1908,7 +2100,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C13">
         <v>6.5</v>
@@ -1920,7 +2112,7 @@
         <v>118</v>
       </c>
       <c r="F13" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G13">
         <v>822941</v>
@@ -1979,17 +2171,23 @@
       <c r="Y13">
         <v>1.0233</v>
       </c>
+      <c r="Z13">
+        <v>9</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB13">
+        <v>0.3</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD13">
         <v>6.8</v>
       </c>
       <c r="AE13" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="AF13">
         <v>0.2911</v>
@@ -1999,6 +2197,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>2.2</v>
+      </c>
+      <c r="AJ13">
+        <v>2.2</v>
+      </c>
+      <c r="AK13">
+        <v>2.2</v>
+      </c>
+      <c r="AL13">
+        <v>2.2</v>
       </c>
       <c r="AM13">
         <v>6.8</v>
@@ -2009,7 +2219,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C14">
         <v>4.5</v>
@@ -2021,13 +2231,13 @@
         <v>-115</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G14">
         <v>824480</v>
       </c>
       <c r="H14" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="I14">
         <v>4</v>
@@ -2080,17 +2290,23 @@
       <c r="Y14">
         <v>1.076</v>
       </c>
+      <c r="Z14">
+        <v>6</v>
+      </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB14">
+        <v>0.41</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD14">
         <v>4.91</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.2119</v>
@@ -2100,6 +2316,18 @@
       </c>
       <c r="AH14">
         <v>0</v>
+      </c>
+      <c r="AI14">
+        <v>1.09</v>
+      </c>
+      <c r="AJ14">
+        <v>1.09</v>
+      </c>
+      <c r="AK14">
+        <v>1.09</v>
+      </c>
+      <c r="AL14">
+        <v>1.09</v>
       </c>
       <c r="AM14">
         <v>4.91</v>
@@ -2110,7 +2338,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C15">
         <v>5.5</v>
@@ -2122,7 +2350,7 @@
         <v>-135</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G15">
         <v>824480</v>
@@ -2181,17 +2409,23 @@
       <c r="Y15">
         <v>0.9392</v>
       </c>
+      <c r="Z15">
+        <v>4</v>
+      </c>
       <c r="AA15" t="s">
         <v>44</v>
       </c>
+      <c r="AB15">
+        <v>-0.76</v>
+      </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD15">
         <v>4.74</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
         <v>0.1804</v>
@@ -2201,6 +2435,18 @@
       </c>
       <c r="AH15">
         <v>0</v>
+      </c>
+      <c r="AI15">
+        <v>-0.74</v>
+      </c>
+      <c r="AJ15">
+        <v>0.74</v>
+      </c>
+      <c r="AK15">
+        <v>-0.74</v>
+      </c>
+      <c r="AL15">
+        <v>0.74</v>
       </c>
       <c r="AM15">
         <v>4.74</v>
@@ -2211,16 +2457,16 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G16">
         <v>824400</v>
       </c>
       <c r="H16" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I16">
         <v>1</v>
@@ -2274,16 +2520,16 @@
         <v>0.88</v>
       </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD16">
         <v>0.4</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.1547</v>
@@ -2303,7 +2549,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C17">
         <v>5.5</v>
@@ -2315,7 +2561,7 @@
         <v>-138</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G17">
         <v>824400</v>
@@ -2374,17 +2620,23 @@
       <c r="Y17">
         <v>1.0658</v>
       </c>
+      <c r="Z17">
+        <v>7</v>
+      </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB17">
+        <v>-0.83</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="AD17">
         <v>4.67</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.2719</v>
@@ -2394,6 +2646,18 @@
       </c>
       <c r="AH17">
         <v>0</v>
+      </c>
+      <c r="AI17">
+        <v>2.33</v>
+      </c>
+      <c r="AJ17">
+        <v>2.33</v>
+      </c>
+      <c r="AK17">
+        <v>2.33</v>
+      </c>
+      <c r="AL17">
+        <v>2.33</v>
       </c>
       <c r="AM17">
         <v>4.67</v>
@@ -2404,7 +2668,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C18">
         <v>4.5</v>
@@ -2416,7 +2680,7 @@
         <v>-104</v>
       </c>
       <c r="F18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G18">
         <v>824157</v>
@@ -2475,17 +2739,23 @@
       <c r="Y18">
         <v>0.9861</v>
       </c>
+      <c r="Z18">
+        <v>8</v>
+      </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB18">
+        <v>-0.12</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD18">
         <v>4.38</v>
       </c>
       <c r="AE18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF18">
         <v>0.2138</v>
@@ -2495,6 +2765,18 @@
       </c>
       <c r="AH18">
         <v>0</v>
+      </c>
+      <c r="AI18">
+        <v>3.62</v>
+      </c>
+      <c r="AJ18">
+        <v>3.62</v>
+      </c>
+      <c r="AK18">
+        <v>3.62</v>
+      </c>
+      <c r="AL18">
+        <v>3.62</v>
       </c>
       <c r="AM18">
         <v>4.38</v>
@@ -2505,7 +2787,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C19">
         <v>4.5</v>
@@ -2517,7 +2799,7 @@
         <v>-135</v>
       </c>
       <c r="F19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G19">
         <v>824157</v>
@@ -2576,17 +2858,23 @@
       <c r="Y19">
         <v>0.9867</v>
       </c>
+      <c r="Z19">
+        <v>6</v>
+      </c>
       <c r="AA19" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB19">
+        <v>-0.47</v>
       </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD19">
         <v>4.03</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.1895</v>
@@ -2596,6 +2884,18 @@
       </c>
       <c r="AH19">
         <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>1.97</v>
+      </c>
+      <c r="AJ19">
+        <v>1.97</v>
+      </c>
+      <c r="AK19">
+        <v>1.97</v>
+      </c>
+      <c r="AL19">
+        <v>1.97</v>
       </c>
       <c r="AM19">
         <v>4.03</v>
@@ -2606,10 +2906,10 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G20">
         <v>823671</v>
@@ -2669,16 +2969,16 @@
         <v>0.9625</v>
       </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD20">
         <v>6.53</v>
       </c>
       <c r="AE20" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="AF20">
         <v>0.3031</v>
@@ -2698,7 +2998,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C21">
         <v>5.5</v>
@@ -2710,7 +3010,7 @@
         <v>-140</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G21">
         <v>823671</v>
@@ -2769,17 +3069,23 @@
       <c r="Y21">
         <v>0.9562</v>
       </c>
+      <c r="Z21">
+        <v>6</v>
+      </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB21">
+        <v>-0.45</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD21">
         <v>5.05</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
         <v>0.2531</v>
@@ -2789,6 +3095,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>0.95</v>
+      </c>
+      <c r="AJ21">
+        <v>0.95</v>
+      </c>
+      <c r="AK21">
+        <v>0.95</v>
+      </c>
+      <c r="AL21">
+        <v>0.95</v>
       </c>
       <c r="AM21">
         <v>5.05</v>
@@ -2799,7 +3117,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C22">
         <v>5.5</v>
@@ -2811,7 +3129,7 @@
         <v>-113</v>
       </c>
       <c r="F22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G22">
         <v>823347</v>
@@ -2870,17 +3188,23 @@
       <c r="Y22">
         <v>1.0844</v>
       </c>
+      <c r="Z22">
+        <v>7</v>
+      </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB22">
+        <v>0.16</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD22">
         <v>5.66</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.218</v>
@@ -2890,6 +3214,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>1.34</v>
+      </c>
+      <c r="AJ22">
+        <v>1.34</v>
+      </c>
+      <c r="AK22">
+        <v>1.34</v>
+      </c>
+      <c r="AL22">
+        <v>1.34</v>
       </c>
       <c r="AM22">
         <v>5.66</v>
@@ -2900,7 +3236,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C23">
         <v>4.5</v>
@@ -2912,7 +3248,7 @@
         <v>106</v>
       </c>
       <c r="F23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G23">
         <v>823347</v>
@@ -2971,17 +3307,23 @@
       <c r="Y23">
         <v>0.9661</v>
       </c>
+      <c r="Z23">
+        <v>7</v>
+      </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB23">
+        <v>-0.48</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD23">
         <v>4.02</v>
       </c>
       <c r="AE23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF23">
         <v>0.2559</v>
@@ -2991,6 +3333,18 @@
       </c>
       <c r="AH23">
         <v>0</v>
+      </c>
+      <c r="AI23">
+        <v>2.98</v>
+      </c>
+      <c r="AJ23">
+        <v>2.98</v>
+      </c>
+      <c r="AK23">
+        <v>2.98</v>
+      </c>
+      <c r="AL23">
+        <v>2.98</v>
       </c>
       <c r="AM23">
         <v>4.02</v>
@@ -3001,7 +3355,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C24">
         <v>4.5</v>
@@ -3013,7 +3367,7 @@
         <v>-149</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G24">
         <v>824884</v>
@@ -3072,17 +3426,23 @@
       <c r="Y24">
         <v>0.9928</v>
       </c>
+      <c r="Z24">
+        <v>5</v>
+      </c>
       <c r="AA24" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB24">
+        <v>0.18</v>
       </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD24">
         <v>4.68</v>
       </c>
       <c r="AE24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF24">
         <v>0.1697</v>
@@ -3092,6 +3452,18 @@
       </c>
       <c r="AH24">
         <v>0</v>
+      </c>
+      <c r="AI24">
+        <v>0.32</v>
+      </c>
+      <c r="AJ24">
+        <v>0.32</v>
+      </c>
+      <c r="AK24">
+        <v>0.32</v>
+      </c>
+      <c r="AL24">
+        <v>0.32</v>
       </c>
       <c r="AM24">
         <v>4.68</v>
@@ -3102,7 +3474,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C25">
         <v>3.5</v>
@@ -3114,7 +3486,7 @@
         <v>115</v>
       </c>
       <c r="F25" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G25">
         <v>824884</v>
@@ -3173,17 +3545,23 @@
       <c r="Y25">
         <v>0.88</v>
       </c>
+      <c r="Z25">
+        <v>3</v>
+      </c>
       <c r="AA25" t="s">
         <v>44</v>
       </c>
+      <c r="AB25">
+        <v>-0.71</v>
+      </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD25">
         <v>2.79</v>
       </c>
       <c r="AE25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF25">
         <v>0.1865</v>
@@ -3193,6 +3571,18 @@
       </c>
       <c r="AH25">
         <v>0</v>
+      </c>
+      <c r="AI25">
+        <v>0.21</v>
+      </c>
+      <c r="AJ25">
+        <v>0.21</v>
+      </c>
+      <c r="AK25">
+        <v>0.21</v>
+      </c>
+      <c r="AL25">
+        <v>0.21</v>
       </c>
       <c r="AM25">
         <v>2.79</v>
@@ -3203,7 +3593,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C26">
         <v>8.5</v>
@@ -3215,7 +3605,7 @@
         <v>-104</v>
       </c>
       <c r="F26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G26">
         <v>823914</v>
@@ -3274,17 +3664,23 @@
       <c r="Y26">
         <v>0.9577</v>
       </c>
+      <c r="Z26">
+        <v>6</v>
+      </c>
       <c r="AA26" t="s">
         <v>44</v>
       </c>
+      <c r="AB26">
+        <v>-0.83</v>
+      </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD26">
         <v>8.44</v>
       </c>
       <c r="AE26" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="AF26">
         <v>0.4022</v>
@@ -3294,6 +3690,18 @@
       </c>
       <c r="AH26">
         <v>-0.77</v>
+      </c>
+      <c r="AI26">
+        <v>-2.44</v>
+      </c>
+      <c r="AJ26">
+        <v>2.44</v>
+      </c>
+      <c r="AK26">
+        <v>-1.67</v>
+      </c>
+      <c r="AL26">
+        <v>1.67</v>
       </c>
       <c r="AM26">
         <v>7.67</v>
@@ -3304,7 +3712,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C27">
         <v>4.5</v>
@@ -3316,7 +3724,7 @@
         <v>134</v>
       </c>
       <c r="F27" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G27">
         <v>823914</v>
@@ -3375,17 +3783,23 @@
       <c r="Y27">
         <v>0.9537</v>
       </c>
+      <c r="Z27">
+        <v>6</v>
+      </c>
       <c r="AA27" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB27">
+        <v>1.27</v>
       </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD27">
         <v>5.77</v>
       </c>
       <c r="AE27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF27">
         <v>0.2066</v>
@@ -3395,6 +3809,18 @@
       </c>
       <c r="AH27">
         <v>0</v>
+      </c>
+      <c r="AI27">
+        <v>0.23</v>
+      </c>
+      <c r="AJ27">
+        <v>0.23</v>
+      </c>
+      <c r="AK27">
+        <v>0.23</v>
+      </c>
+      <c r="AL27">
+        <v>0.23</v>
       </c>
       <c r="AM27">
         <v>5.77</v>
@@ -3405,7 +3831,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C28">
         <v>3.5</v>
@@ -3417,7 +3843,7 @@
         <v>-150</v>
       </c>
       <c r="F28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G28">
         <v>823990</v>
@@ -3476,17 +3902,23 @@
       <c r="Y28">
         <v>1.0238</v>
       </c>
+      <c r="Z28">
+        <v>6</v>
+      </c>
       <c r="AA28" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB28">
+        <v>-0.7</v>
       </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="AD28">
         <v>2.8</v>
       </c>
       <c r="AE28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF28">
         <v>0.1277</v>
@@ -3496,6 +3928,18 @@
       </c>
       <c r="AH28">
         <v>0</v>
+      </c>
+      <c r="AI28">
+        <v>3.2</v>
+      </c>
+      <c r="AJ28">
+        <v>3.2</v>
+      </c>
+      <c r="AK28">
+        <v>3.2</v>
+      </c>
+      <c r="AL28">
+        <v>3.2</v>
       </c>
       <c r="AM28">
         <v>2.8</v>
@@ -3506,7 +3950,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C29">
         <v>6.5</v>
@@ -3518,7 +3962,7 @@
         <v>-132</v>
       </c>
       <c r="F29" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G29">
         <v>823990</v>
@@ -3577,17 +4021,23 @@
       <c r="Y29">
         <v>0.9579</v>
       </c>
+      <c r="Z29">
+        <v>11</v>
+      </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB29">
+        <v>-0.94</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="AD29">
         <v>5.56</v>
       </c>
       <c r="AE29" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF29">
         <v>0.2958</v>
@@ -3597,6 +4047,18 @@
       </c>
       <c r="AH29">
         <v>0</v>
+      </c>
+      <c r="AI29">
+        <v>5.44</v>
+      </c>
+      <c r="AJ29">
+        <v>5.44</v>
+      </c>
+      <c r="AK29">
+        <v>5.44</v>
+      </c>
+      <c r="AL29">
+        <v>5.44</v>
       </c>
       <c r="AM29">
         <v>5.56</v>
@@ -3607,7 +4069,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C30">
         <v>6.5</v>
@@ -3619,7 +4081,7 @@
         <v>-138</v>
       </c>
       <c r="F30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G30">
         <v>824966</v>
@@ -3678,17 +4140,23 @@
       <c r="Y30">
         <v>1.057</v>
       </c>
+      <c r="Z30">
+        <v>5</v>
+      </c>
       <c r="AA30" t="s">
         <v>44</v>
       </c>
+      <c r="AB30">
+        <v>-0.01</v>
+      </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD30">
         <v>6.49</v>
       </c>
       <c r="AE30" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="AF30">
         <v>0.268</v>
@@ -3698,6 +4166,18 @@
       </c>
       <c r="AH30">
         <v>0</v>
+      </c>
+      <c r="AI30">
+        <v>-1.49</v>
+      </c>
+      <c r="AJ30">
+        <v>1.49</v>
+      </c>
+      <c r="AK30">
+        <v>-1.49</v>
+      </c>
+      <c r="AL30">
+        <v>1.49</v>
       </c>
       <c r="AM30">
         <v>6.49</v>
@@ -3708,10 +4188,10 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F31" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G31">
         <v>824966</v>
@@ -3771,16 +4251,16 @@
         <v>1.1186</v>
       </c>
       <c r="AA31" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD31">
         <v>5.83</v>
       </c>
       <c r="AE31" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF31">
         <v>0.2131</v>
@@ -3800,7 +4280,7 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32">
         <v>6.5</v>
@@ -3812,31 +4292,31 @@
         <v>-120</v>
       </c>
       <c r="F32" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G32" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H32" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L32">
         <v>6</v>
       </c>
       <c r="S32" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="V32" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AA32" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AC32" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AE32" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:39" x14ac:dyDescent="0.25">
@@ -3844,7 +4324,7 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C33">
         <v>4.5</v>
@@ -3856,31 +4336,31 @@
         <v>-103</v>
       </c>
       <c r="F33" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G33" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H33" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L33">
         <v>6</v>
       </c>
       <c r="S33" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="V33" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AA33" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AC33" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AE33" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>